<commit_message>
La til noen grafer i excel
mulig jeg fucket opp csv filene, hvis det har skjedd er det her. lagde noen modeller
</commit_message>
<xml_diff>
--- a/data/spool_mapping/mapping.xlsx
+++ b/data/spool_mapping/mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sujro\Documents\GitHub\Bachelor\data\spool_mapping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1A633B7-3833-4BDD-BA50-F733917AE8E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08AFAC22-F3C6-419D-92EE-56D905AD7CD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{AD92D090-37B1-4D85-9043-B221BBD43E04}"/>
   </bookViews>
@@ -143,7 +143,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -168,7 +168,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4510,8 +4509,8 @@
       <xdr:row>82</xdr:row>
       <xdr:rowOff>151328</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="12" name="Ink 11">
@@ -4530,7 +4529,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="12" name="Ink 11">
@@ -4575,8 +4574,8 @@
       <xdr:row>82</xdr:row>
       <xdr:rowOff>122168</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="18" name="Ink 17">
@@ -4595,7 +4594,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="18" name="Ink 17">
@@ -4640,8 +4639,8 @@
       <xdr:row>73</xdr:row>
       <xdr:rowOff>16815</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="19" name="Ink 18">
@@ -4660,7 +4659,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="19" name="Ink 18">
@@ -4705,8 +4704,8 @@
       <xdr:row>94</xdr:row>
       <xdr:rowOff>50358</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="26" name="Ink 25">
@@ -4725,7 +4724,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="26" name="Ink 25">
@@ -4770,8 +4769,8 @@
       <xdr:row>92</xdr:row>
       <xdr:rowOff>16187</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="27" name="Ink 26">
@@ -4790,7 +4789,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="27" name="Ink 26">
@@ -4835,8 +4834,8 @@
       <xdr:row>96</xdr:row>
       <xdr:rowOff>152570</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId14">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="33" name="Ink 32">
@@ -4855,7 +4854,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="33" name="Ink 32">
@@ -4900,8 +4899,8 @@
       <xdr:row>82</xdr:row>
       <xdr:rowOff>152048</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId16">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="43" name="Ink 42">
@@ -4920,7 +4919,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="43" name="Ink 42">
@@ -4965,8 +4964,8 @@
       <xdr:row>94</xdr:row>
       <xdr:rowOff>138918</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId18">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="44" name="Ink 43">
@@ -4985,7 +4984,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="44" name="Ink 43">
@@ -5030,8 +5029,8 @@
       <xdr:row>95</xdr:row>
       <xdr:rowOff>51064</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId20">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="47" name="Ink 46">
@@ -5050,7 +5049,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="47" name="Ink 46">
@@ -5154,6 +5153,266 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>371213</xdr:colOff>
+      <xdr:row>88</xdr:row>
+      <xdr:rowOff>3067</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>509993</xdr:colOff>
+      <xdr:row>98</xdr:row>
+      <xdr:rowOff>22837</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId24">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="3" name="Ink 2">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1805953F-977D-D906-A3E0-B25D8C87C69A}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="4705088" y="16009830"/>
+            <a:ext cx="2767680" cy="1829520"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="3" name="Ink 2">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1805953F-977D-D906-A3E0-B25D8C87C69A}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId25"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4698966" y="16003798"/>
+              <a:ext cx="2779923" cy="1841584"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>479408</xdr:colOff>
+      <xdr:row>79</xdr:row>
+      <xdr:rowOff>172042</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>95453</xdr:colOff>
+      <xdr:row>94</xdr:row>
+      <xdr:rowOff>162457</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId26">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="17" name="Ink 16">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{87974995-DA1C-13FE-33CF-B39927D5D537}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="479408" y="14550030"/>
+            <a:ext cx="3949920" cy="2705040"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="17" name="Ink 16">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{87974995-DA1C-13FE-33CF-B39927D5D537}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId27"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="473271" y="14543984"/>
+              <a:ext cx="3962194" cy="2717132"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1962060</xdr:colOff>
+      <xdr:row>94</xdr:row>
+      <xdr:rowOff>141577</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>319373</xdr:colOff>
+      <xdr:row>95</xdr:row>
+      <xdr:rowOff>124042</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId28">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="20" name="Ink 19">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BB366706-0970-BADF-33BB-548FDAD298A4}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="4300448" y="17234190"/>
+            <a:ext cx="352800" cy="163440"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="20" name="Ink 19">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BB366706-0970-BADF-33BB-548FDAD298A4}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId29"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4294328" y="17228070"/>
+              <a:ext cx="365040" cy="175680"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>561848</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>55927</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>689948</xdr:colOff>
+      <xdr:row>87</xdr:row>
+      <xdr:rowOff>82</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId30">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="23" name="Ink 22">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{42493182-86B6-8B21-AF24-E155D70BF641}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="561848" y="15338790"/>
+            <a:ext cx="775800" cy="487080"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="23" name="Ink 22">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{42493182-86B6-8B21-AF24-E155D70BF641}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId31"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="555728" y="15332670"/>
+              <a:ext cx="788040" cy="499320"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -5180,11 +5439,128 @@
       <inkml:brushProperty name="height" value="0.035" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">34 284 24575,'0'531'0,"-2"-505"0,0 0 0,-10 40 0,5-35 0,-2 38 0,7 203-790,4-140 780,-2-101-95,2 82 330,0-94-563,0-1 0,2 1 0,10 35 0,-1-20-5821</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1239.84">34 284 24575,'1'0'0,"0"-1"0,0 1 0,0-1 0,1 1 0,-1-1 0,0 1 0,0-1 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0-2 0,4-4 0,7-9 0,1 1 0,0 0 0,1 1 0,1 0 0,0 1 0,1 1 0,0 0 0,1 2 0,19-11 0,21-4-995,98-30 0,-115 43 995,-23 6 0,1 1 0,0 1 0,18-2 0,7 3 663,-1 1 1,55 6-1,-91-3-663,0-1 0,-1 1 0,1 1 0,-1-1 0,0 1 0,1 0 0,-1 0 0,0 1 0,0-1 0,0 1 0,8 6 0,-5-1 0,0 1 0,0-1 0,0 1 0,9 15 0,12 18 0,-2 1 0,26 56 0,-47-84 0,-1 1 0,6 27 0,1 5 0,-6-28 0,-2 1 0,0 0 0,-1 1 0,-1-1 0,-1 1 0,0-1 0,-2 1 0,-7 39 0,4-46 0,0 1 0,-2-1 0,0-1 0,-1 1 0,0-1 0,-1 0 0,0 0 0,-15 17 0,-12 10 0,-45 41 0,61-64 0,14-13 0,0 0 0,-1 0 0,0 0 0,0-1 0,0 0 0,-8 5 0,11-8 0,1 0 0,-1-1 0,1 1 0,-1 0 0,1-1 0,-1 0 0,1 1 0,-1-1 0,0 0 0,1 0 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,-2-2 0,-7-6 0,1 0 0,0-1 0,0 0 0,1-1 0,-12-16 0,-9-9 0,-130-125 0,147 146 0,-2-2 0,-1 1 0,-28-23 0,38 35 25,0 0 0,0 1 0,-12-5 0,-6-2-1490,8 1-5361</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2004.27">563 1623 24575,'5'-1'0,"0"1"0,0-1 0,0 0 0,-1 0 0,1 0 0,0-1 0,0 0 0,-1 0 0,7-4 0,6-4 0,16-14 0,-9 6 0,91-55-1071,22-17-344,1-4 1415,30-22 0,-138 95 0,40-20 0,11-7 0,5-6 78,25-18 44,-110 71-123,0 1-1,0-1 0,0 0 0,-1 1 1,1-1-1,0 1 0,0-1 1,0 1-1,0-1 0,0 1 1,0 0-1,0-1 0,0 1 1,1 0-1,-1 0 0,1 0 0,-1 0 4,0 0 0,-1 0 0,1 0 0,-1 1 0,1-1 0,-1 0-1,0 1 1,1-1 0,-1 0 0,1 1 0,-1-1 0,1 1 0,-1-1 0,0 0-1,1 1 1,-1-1 0,0 1 0,0-1 0,1 1 0,-1-1 0,0 1 0,0 0-1,2 5 172,-2-1-1,1 1 0,-1-1 0,1 1 1,-2 6-1,1-5 325,1 17-286,1 0 0,8 34-1,2 31-101,-10 205-109,-3-153 0,1-122 0,0 7 0,5 47 0,-3-54-1365,-2-6-5461</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2604.23">968 1404 24575,'3'3'0,"0"-1"0,1 1 0,-1-1 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 0 0,6 1 0,8 1 0,24 0 0,-34-2 0,160 1-128,-111-3-1935,-23-2 1732,0-1-1,0-1 1,66-21 0,-25 6 207,-29 8 34,-18 5-81,58-9 0,-50 11 691,-1-1 0,1-2 1,41-15-1,-50 14-6720</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="3653.18">1963 1778 24575,'0'-18'0,"0"-3"0,0 0 0,4-21 0,-3 35 0,1-1 0,0 1 0,0 0 0,1 0 0,0 1 0,0-1 0,0 0 0,1 1 0,7-10 0,-3 7 0,1-1 0,0 1 0,1 1 0,0-1 0,1 2 0,-1-1 0,2 2 0,-1-1 0,0 2 0,1-1 0,0 2 0,17-5 0,1-2 0,-22 7 0,0 1 0,1 1 0,0-1 0,-1 1 0,14-1 0,-19 3 0,-1 0 0,1 0 0,0 0 0,0 1 0,-1-1 0,1 1 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 1 0,1-1 0,-1 1 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,-1 0 0,3 4 0,1 1 0,-1 1 0,1 0 0,-2 0 0,1 0 0,-1 1 0,0-1 0,-1 1 0,0 0 0,0 0 0,-1 0 0,0 0 0,-1 0 0,-1 14 0,0-10 0,-1 0 0,0 0 0,-1-1 0,0 1 0,-1-1 0,-1 0 0,0 0 0,-13 23 0,5-15 0,-2-1 0,0 0 0,-20 20 0,-57 45 0,76-72 0,-26 16 0,29-21 0,1 1 0,0 0 0,0 1 0,-19 19 0,28-24 0,1-1 0,-1 1 0,1-1 0,0 1 0,-1 0 0,2 0 0,-1 0 0,0 0 0,1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,1 0 0,0 1 0,0-1 0,0 1 0,0-1 0,1 0 0,1 8 0,-1-7 0,1-1 0,0 1 0,0 0 0,0-1 0,0 1 0,1-1 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1-1 0,1 0 0,0 1 0,7 3 0,6 4 0,1-2 0,31 12 0,-43-18 0,3 1 0,1-1 0,0 0 0,0-1 0,0 0 0,0 0 0,0-1 0,0-1 0,0 1 0,0-2 0,0 1 0,1-2 0,-1 1 0,0-1 0,0-1 0,-1 1 0,1-2 0,-1 1 0,13-8 0,288-142 0,-263 129 92,10-6-1549,-35 22-5369</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">34 290 24575,'0'542'0,"-2"-515"0,0-1 0,-10 42 0,5-37 0,-2 40 0,7 207-790,4-144 780,-2-102-95,2 83 330,0-95-563,0-2 0,2 2 0,10 35 0,-1-21-5821</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1239.83">34 290 24575,'1'0'0,"0"-1"0,0 1 0,0-1 0,1 1 0,-1-1 0,0 1 0,0-1 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0-2 0,4-5 0,7-8 0,1 1 0,0 0 0,1 0 0,1 1 0,0 1 0,1 0 0,0 1 0,1 2 0,19-12 0,21-3-995,98-31 0,-115 44 995,-23 5 0,1 2 0,0 1 0,18-2 0,7 3 663,-1 1 1,55 6-1,-91-3-663,0-1 0,-1 1 0,1 1 0,-1-1 0,0 1 0,1 0 0,-1 0 0,0 1 0,0-1 0,0 1 0,8 7 0,-5-2 0,0 1 0,0-1 0,0 1 0,9 16 0,12 18 0,-2 1 0,26 57 0,-47-86 0,-1 1 0,6 28 0,1 5 0,-6-28 0,-2 0 0,0 1 0,-1 0 0,-1 0 0,-1 0 0,0-1 0,-2 2 0,-7 39 0,4-46 0,0 0 0,-2-1 0,0-1 0,-1 2 0,0-2 0,-1 0 0,0 1 0,-15 16 0,-12 11 0,-45 42 0,61-66 0,14-13 0,0 1 0,-1-1 0,0 0 0,0-1 0,0 0 0,-8 5 0,11-8 0,1 0 0,-1-1 0,1 1 0,-1 0 0,1-1 0,-1 0 0,1 1 0,-1-1 0,0 0 0,1 0 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,-2-2 0,-7-6 0,1 0 0,0-2 0,0 1 0,1-1 0,-12-17 0,-9-8 0,-130-129 0,147 150 0,-2-2 0,-1 0 0,-28-23 0,38 36 25,0 0 0,0 1 0,-12-5 0,-6-2-1490,8 1-5361</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2004.27">563 1657 24575,'5'-1'0,"0"1"0,0-1 0,0 0 0,-1 0 0,1 0 0,0-1 0,0 0 0,-1 0 0,7-4 0,6-4 0,16-15 0,-9 7 0,91-57-1071,22-17-344,1-4 1415,30-22 0,-138 96 0,40-19 0,12-8 0,4-7 78,25-17 44,-110 72-123,0 1-1,0-1 0,0 0 0,-1 1 1,1-1-1,0 1 0,0-1 1,0 1-1,0-1 0,0 1 1,0 0-1,0-1 0,0 1 1,1 0-1,-1 0 0,1 0 0,-1 0 4,0 0 0,-1 0 0,1 0 0,-1 1 0,1-1 0,-1 0-1,0 1 1,1-1 0,-1 0 0,1 1 0,-1-1 0,1 1 0,-1-1 0,0 0-1,1 1 1,-1-1 0,0 1 0,0-1 0,1 1 0,-1-1 0,0 1 0,0 0-1,2 5 172,-2-1-1,1 1 0,-1-1 0,1 2 1,-2 5-1,1-5 325,1 17-286,1 1 0,8 34-1,2 32-101,-10 209-109,-3-156 0,1-124 0,0 6 0,5 49 0,-3-56-1365,-2-6-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2604.23">968 1434 24575,'3'3'0,"0"-1"0,1 1 0,-1-1 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 0 0,6 1 0,8 1 0,24 0 0,-34-2 0,160 1-128,-111-3-1935,-23-2 1732,1-1-1,-1-1 1,66-22 0,-25 7 207,-29 8 34,-18 5-81,58-10 0,-50 12 691,-1-1 0,1-2 1,41-16-1,-50 15-6720</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="3653.18">1964 1815 24575,'0'-18'0,"0"-3"0,0-1 0,4-21 0,-3 36 0,1-1 0,0 1 0,0 0 0,1 0 0,0 0 0,0 0 0,0 0 0,1 1 0,7-10 0,-3 6 0,1 0 0,0 1 0,1 1 0,0-1 0,1 2 0,-1-2 0,2 3 0,-1-1 0,0 2 0,1-1 0,0 2 0,17-5 0,1-3 0,-22 8 0,0 1 0,1 1 0,0-1 0,-1 1 0,14-1 0,-19 3 0,-1 0 0,1 0 0,0 0 0,0 1 0,-1-1 0,1 1 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 1 0,1-1 0,-1 1 0,0 0 0,0-1 0,0 1 0,0 0 0,0 1 0,-1-1 0,3 4 0,1 1 0,-1 1 0,1 0 0,-2 0 0,1 1 0,-1 0 0,0-1 0,-1 1 0,0 0 0,0 0 0,-1 1 0,0-1 0,-1 0 0,-1 14 0,0-9 0,-1-1 0,0 0 0,-1 0 0,0 0 0,-1-1 0,-1 0 0,0 1 0,-13 22 0,5-14 0,-2-2 0,0 1 0,-20 19 0,-57 47 0,76-74 0,-26 17 0,29-22 0,1 1 0,0 0 0,0 2 0,-19 18 0,28-24 0,1-1 0,-1 1 0,1 0 0,0 0 0,-1 0 0,2 0 0,-1 0 0,0 0 0,1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,1 1 0,0 0 0,0-1 0,0 1 0,0-1 0,1 0 0,1 8 0,-1-7 0,1-1 0,0 2 0,0-1 0,0-1 0,0 1 0,1-1 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1-1 0,1 0 0,0 2 0,7 2 0,6 4 0,1-2 0,31 13 0,-43-19 0,3 1 0,1-1 0,0 0 0,0-1 0,0 0 0,0 0 0,0-1 0,0-1 0,0 1 0,0-2 0,0 1 0,1-2 0,-1 1 0,0-1 0,0-1 0,-1 1 0,1-2 0,-1 1 0,13-9 0,288-144 0,-263 132 92,10-7-1549,-35 23-5369</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink10.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-19T11:15:10.108"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#E71224"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 3750 24575,'0'6'0,"0"0"0,0 0 0,1 0 0,0 0 0,2 8 0,2 5 0,17 68-328,4-2 1,4 0-1,44 88 0,-43-113 240,2-1 0,2-1 0,3-2 0,3-2-1,2-1 1,1-3 0,3-1 0,3-3 0,1-2 0,1-2 0,3-3 0,1-2 0,2-2 0,1-3 0,108 41-1,-84-44 24,0-4 0,1-4 0,2-3-1,0-4 1,139 5 0,-172-21-74,-1-1-1,0-3 1,0-3 0,0-1-1,97-34 1,-36 0-551,153-84-1,113-101 330,-294 169 643,-2-5 0,90-90 0,-146 127-214,-1-1 0,-1-1 0,-1-2 0,-2 0 0,-1-1 0,-1-1 0,-2-1 1,-2-1-1,14-43 0,22-114-228,-6-54-902,-2-46 468,35-387-776,-11-1088 0,-70 1723 1496,2-25 1528,0 67-1463,0 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,1 1 0,-1-1 0,1 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,5-3 0,19-17 975,53-35 1,39-13-346,-72 43-989,126-68-166,355-140 1,-400 191 250,187-39-1,-210 64 95,1 5 0,143-2 0,-212 15-14,-1 3-1,1 0 0,0 3 0,-1 1 0,1 1 0,-2 3 1,1 0-1,41 20 0,64 45-69,15 8 1082,-148-80-999,0 0 1,0 0 0,1-1-1,-1 0 1,1-1-1,-1 1 1,1-1 0,-1-1-1,1 0 1,0 0 0,-1 0-1,1-1 1,0 0 0,-1 0-1,1-1 1,-1 0 0,0-1-1,0 1 1,0-1 0,8-5-1,-14 8-10,81-39 0,-70 34 0,1 1 0,-1 1 0,1 0 0,-1 1 0,15-1 0,95 2 0,-105 2 0,-1 1 0,1 0 0,-1 2 0,1 0 0,18 8 0,-10 2 0,-21-11 0,1 0 0,0 0 0,0-1 0,8 4 0,189 70 0,-128-45 0,79 21 0,-150-51 0,114 25 0,-103-25 0,-1 1 0,0-2 0,0 0 0,0 0 0,0-2 0,1 1 0,12-5 0,-10 3-60,0 1 0,0 0 0,-1 1 0,24 2 1,-17-1-1007,-5 0-5760</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink11.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-19T11:15:24.850"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#E71224"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">7365 1230 24575,'-50'1'0,"-72"3"0,-84 2-1077,-69-1-3233,-908-6-55,-8-63 1866,872 33 2330,-533-38 596,610 61 1724,-368 36 0,343 9 4822,257-34-7764,4 0-5891</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2410.03">2036 172 24575,'0'38'82,"3"564"-3184,19-5 1899,-21-583 1204,40 502 164,-21-352-85,47 182-1,69 329-79,-125-599 32,69 515 835,-75-555-368,-1-12 334,-2-1 1,0 37-1,-27 196-833,-1 7 0,26-248 0,1 1 0,1-1 0,0 1 0,1-1 0,0 0 0,7 17 0,-2-5 0,-6-22 0,0 1 0,-1 0 0,1 1 0,-1-1 0,0 0 0,0 12 0,-1-17 0,0 1 0,0-1 0,0 0 0,-1 0 0,1 1 0,0-1 0,-1 0 0,1 0 0,-1 1 0,0-1 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,-1-1 0,1 1 0,0 0 0,0-1 0,0 0 0,-1 1 0,1-1 0,0 0 0,-1 0 0,1 1 0,-2-1 0,-32 1 0,0-1 0,-39-6 0,-29 0 0,-166 21 0,2 22 0,-25 2 0,196-30 0,-103-5 0,122-6 0,74 2 0,0-1 0,0 1 0,0 0 0,1-1 0,-1 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1-1 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 1 0,0-1 0,0-1 0,-2-2 0,-13-14 0,1-1 0,1 0 0,-15-29 0,-33-74 0,-79-229-1097,113 277 1000,-33-97-588,8-2 1,-36-194-1,9-225-1146,44-7-592,13-257 1711,8 634 1431,8 164 1814,-26-99 0,20 112-1048,-18-75-485,26 93-1019,1 0 1,-1-41-1,6 66 19,0-1 0,0 1 0,0-1 0,0 1 0,1 0 0,0-1 0,-1 1 0,3-5 0,-2 6 0,0 0 0,0 1 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,1 0 0,-1-1 0,0 1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 1 0,0-1 0,-1 0 0,4 0 0,6-2 0,1 1 0,0 1 0,-1 0 0,13 1 0,-16-1 0,120-4-542,207-37 0,-92-9-571,295-103-1,146-104 387,-674 253 943,-2 2-19,0 0-1,-1 0 1,10-2-1,-15 4-94,-1 1-1,1 0 1,0 0-1,-1-1 1,1 1-1,0 0 1,-1 0-1,1 1 1,0-1-1,-1 0 0,1 1 1,-1-1-1,1 1 1,0-1-1,-1 1 1,1 0-1,-1-1 1,1 1-1,-1 0 0,3 2 1,-2-1 23,-2-1-151,0-1 1,1 1 0,-1-1-1,0 0 1,0 1-1,1-1 1,-1 0-1,1 1 1,-1-1 0,0 0-1,1 1 1,-1-1-1,1 0 1,-1 0-1,1 1 1,-1-1 0,0 0-1,1 0 1,-1 0-1,1 0 1,-1 0-1,2 0 1</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="5925.49">10941 7605 24575,'-42'-36'0,"-70"-58"0,-94-75-1638,-97-76-4918,-77-67 4425,-524-454-701,-281-230 288,832 713 2179,42 40 415,37 41 151,32 35 52,-567-349 1960,587 378-885,188 118-1277,19 12 990,1 0 1,0-1-1,1-1 1,0 0 0,0 0-1,-16-19 1,34 33-39,1 2-84,1 1 0,-1 0 0,10 14 0,-47-49-919,-73-71 0,4 5 0,65 53 0,1-1 0,-33-56 0,-47-99 0,61 102 0,36 65 0,-36-47 0,41 63 0,0 1 0,0 0 0,-1 1 0,-1 1 0,-15-11 0,11 9 0,-30-14 0,40 24 0,1 0 0,-1 0 0,0 0 0,0 1 0,-1 1 0,1-1 0,-10 1 0,6 0 0,0 0 0,-17-3 0,25 3 0,-1-1 0,0 1 0,1-1 0,0 0 0,-1 0 0,1-1 0,0 1 0,0-1 0,-4-3 0,-8-6 0,0 0 0,-35-17 0,-4-2 0,23 7 0,1-1 0,1-2 0,-45-52 0,10 10 0,38 43 0,-1 1 0,-1 1 0,-1 1 0,-44-24 0,55 36 0,-1 1 0,0 2 0,-1 0 0,0 1 0,0 1 0,-1 0 0,1 2 0,-38-2 0,10 6 0,-52 8 0,66-4 0,1-1 0,-1-2 0,1-2 0,-39-5 0,45 2 0,-49-10 0,-85-3 0,42 14 0,-149-11 0,93-19 0,162 31 0,-1 0 0,0 1 0,-20 2 0,17-1 0,-25-2 0,36 1 0,1 0 0,0 0 0,0-1 0,0 0 0,0 0 0,1 0 0,-1-1 0,-5-3 0,-11-10 0,18 13 0,0 0 0,0-1 0,0 2 0,-1-1 0,0 0 0,1 1 0,-1 0 0,0 0 0,-8-1 0,-12 0 39,-1 1-1,1 1 0,-28 3 0,-4 0-1556,44-2-5308</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="7057.3">268 1056 24575,'63'36'0,"61"35"0,52 22 0,23 13-5476,5 1 5476,-13-9 0,-18-13-717,-29-19 717,-24-11 673,-31-13-673,-24-11 0,-18-11 0,-14-6 2519,-11-6-2519,-7-5 2120,-5-1-9430</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="7961.18">1930 1070 24575,'-22'11'0,"-39"25"0,-43 33 0,-33 39 0,-31 31-3998,-27 32 3998,-8 15-2947,-3 6 2947,7-8 0,19-19 0,20-19 0,31-23 224,30-30-224,32-32-1470</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink12.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-19T11:15:37.959"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#E71224"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">979 453 24575,'-18'-20'0,"0"-1"0,-20-33 0,4 4 0,23 36 0,-14-19 0,-37-38 0,61 69 0,-1 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,-1 1 0,1-1 0,-1 1 0,1 0 0,-5 0 0,0 1 0,-1 1 0,1 0 0,0 0 0,-12 5 0,-4 1 0,-1-1 0,0-1 0,0-2 0,0 0 0,-29 0 0,12-4 0,-69-8 0,95 6 0,-54-9 0,62 10 0,0-1 0,0 0 0,1-1 0,-1 1 0,0-1 0,1-1 0,-8-5 0,13 9 0,0-1 0,0 1 0,1-1 0,-1 1 0,0-1 0,1 0 0,-1 1 0,1-1 0,-1 0 0,1 1 0,-1-1 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,1-2 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,1 1 0,2-4 0,-2 4 0,0-1 0,-1 1 0,1-1 0,-1 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0-3 0,-1 5 0,0 0 0,0-1 0,0 1 0,0 0 0,-1-1 0,1 1 0,-1 0 0,1 0 0,-1-1 0,1 1 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 0 0,-3 0 0,-3-1 0,-1-1 0,1 2 0,-13-3 0,5 2 0,-14-6-455,0-2 0,-40-18 0,48 19-6371</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink13.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-20T09:25:52.233"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#E71224"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 480 24575,'3'0'0,"-1"0"0,1 0 0,0-1 0,0 1 0,-1-1 0,1 1 0,0-1 0,-1 0 0,1 0 0,0 0 0,-1 0 0,0-1 0,1 1 0,2-3 0,5-2 0,0 0 0,13-5 0,192-71-1156,-83 33-3341,-79 29 3426,108-40-2442,-119 47 2614,81-15 1,78-9 3842,-154 28-2640,-18 5 1080,45-1 0,-46 4 128,53-9 0,-19-5-1205,-30 6 83,1 2 1,52-4-1,-65 8-7,40-8 1,-39 7-10,37-5 1,-44 8-375,1-1 0,-1-1 0,0 0 0,0-1 0,0-1 0,24-12 0,-24 13-170,0 0-1,0 0 0,0 1 1,0 1-1,0 0 0,1 1 1,25 1-1,-18 0-6655</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1679.34">159 1353 24575,'15'0'0,"1"-1"0,-1 0 0,0-2 0,0 1 0,0-2 0,0 0 0,15-7 0,33-9 0,-41 14 0,-1-1 0,30-14 0,96-43 0,72-36 0,-189 86 0,126-72 0,-152 84 0,72-51 0,-51 35 0,7-8 0,53-55 0,-80 77 0,1-1 0,0 1 0,0 0 0,0 0 0,1 0 0,-1 1 0,1 0 0,14-4 0,-2 1 0,41-5 0,-1 7 0,-41 4 0,0-1 0,-1-1 0,22-6 0,-9 2 0,0 2 0,0 1 0,1 1 0,50 3 0,44-3 0,-119 2 0,0-1 0,-1 0 0,1-1 0,-1 1 0,0-1 0,1 0 0,-1-1 0,7-3 0,1-3 0,20-17 0,-1 1 0,-5 5 0,59-31 0,-81 48-53,0 0-1,0 0 1,0-1-1,-1 0 1,0 0-1,5-4 0,-3 1-936,6-4-5836</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -5211,11 +5587,11 @@
       <inkml:brushProperty name="height" value="0.035" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">222 221 24575,'1'69'0,"-3"80"0,-2-115 0,-2 0 0,-14 42 0,11-42 0,-11 71 0,16-81-333,-1 0 0,-1 0 0,-11 29 1,9-30 275,1 2 1,1-1-1,-4 26 1,-6 36-832,10-61 1167,-5 53 0,-4 30-307,8-72 199,-1 37 0,6 20 37,2-66-7034</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="691.44">66 66 24575,'2'-1'0,"1"1"0,-1-1 0,1 1 0,-1-1 0,1 0 0,-1 0 0,0 0 0,4-3 0,12-5 0,46-3 0,2-2 0,-42 8 0,2 1 0,-1 1 0,37-1 0,79 6 0,-61 0 0,-19-1 0,64 1 0,-118 0 0,0 0 0,-1 1 0,1-1 0,-1 1 0,1 1 0,-1-1 0,0 1 0,0 0 0,0 0 0,11 8 0,-2 2 0,0 1 0,17 20 0,-25-27 0,5 8 0,0 1 0,-1 1 0,12 24 0,10 15 0,-27-45 0,0 0 0,0 1 0,-2 0 0,1 0 0,-2 0 0,1 0 0,-2 0 0,3 22 0,7 22 0,-7-35 0,4 31 0,-5 0 0,-2 0 0,-7 58 0,4-100 0,-2 0 0,1 0 0,-1-1 0,-1 1 0,0-1 0,0 1 0,-1-1 0,-11 15 0,11-16 0,1-1 0,-1-1 0,0 0 0,0 0 0,-1-1 0,1 0 0,-1 0 0,0 0 0,-8 4 0,-5 2 0,-33 15 0,24-16 0,1-1 0,-1-1 0,-56 8 0,30-11 0,-88-3 0,87-3 0,28-2-338,0 0-1,0-2 0,0-1 1,-37-13-1,-12-2-162,33 9 429,-39-7 509,1-1 1283,57 14-2976,3 1-5570</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1579.38">720 1622 24575,'0'-13'0,"0"0"0,1 0 0,0 0 0,1 0 0,0 0 0,1 1 0,1-1 0,0 1 0,1 0 0,10-20 0,-1 10 0,31-38 0,-9 13 0,-20 27 0,0 1 0,2 0 0,30-25 0,65-43 0,-107 83 0,139-86-685,-108 68 781,87-40-96,-122 61 14,1-1-1,0 1 1,0-1 0,0 1 0,-1 0-1,1 0 1,0 1 0,0-1-1,4 0 1,-6 1 3,0 0 1,1 0-1,-1 1 0,0-1 1,0 0-1,0 1 1,1-1-1,-1 1 0,0-1 1,0 1-1,0 0 1,0-1-1,0 1 0,0 0 1,0 0-1,0 0 1,0-1-1,-1 1 0,1 0 1,0 0-1,0 0 1,-1 1-1,1-1 0,-1 0 1,2 2-1,4 13-17,0 0 0,0 1 0,-2-1 0,0 1 0,0 0 0,0 23 0,-2 108 0,-3-98 0,0-33 0,-1 0 0,-1-1 0,-7 24 0,5-18 0,-4 25 0,-7 34 0,10-57 0,2 1 0,-3 28 0,5-18 0,3 42 0,1-65 0,-1 0 0,1 0 0,1 0 0,0-1 0,1 1 0,0-1 0,7 14 0,2 2 0,9 28 0,-13-29 0,23 41 0,-22-49 0,-3-5 0,-1-1 0,2 0 0,0-1 0,0 0 0,19 19 0,-27-29 0,0-1 0,1 1 0,-1-1 0,1 1 0,0 0 0,-1-1 0,1 0 0,-1 1 0,1-1 0,0 1 0,-1-1 0,1 0 0,0 1 0,-1-1 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 1 0,0-1 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1-1 0,1 1 0,0 0 0,-1 0 0,1 0 0,0-1 0,0 1 0,0-1 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0-1 0,0 1 0,-1-2 0,-6-34 0,-16-52 0,-9-9 0,16 55-64,4 6-586,-21-39-1,24 58-6175</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2028.66">875 1280 24575,'11'1'0,"-1"0"0,1 1 0,-1 1 0,0 0 0,11 4 0,2 1 0,73 24 0,-18-1 0,2 1 0,-49-22-341,0-2 0,0-2-1,55 6 1,-59-11-6485</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2525.38">1778 1280 24575,'0'26'0,"0"-2"0,0-1 0,-1 1 0,-1-1 0,-7 29 0,2-22 13,1 1 1,-2 58-1,8 64-208,2-67-1015,-2-59-5616</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">222 226 24575,'1'71'0,"-3"81"0,-2-117 0,-2-1 0,-14 44 0,11-43 0,-11 72 0,16-82-333,-1-1 0,-1 1 0,-11 29 1,9-30 275,1 1 1,1 0-1,-4 26 1,-6 37-832,10-63 1167,-5 55 0,-4 31-307,8-75 199,-1 39 0,6 20 37,2-67-7034</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="691.44">66 67 24575,'2'-1'0,"1"1"0,-1-1 0,1 1 0,-1-1 0,1 0 0,-1 0 0,0 0 0,4-3 0,12-5 0,46-3 0,2-3 0,-42 9 0,2 1 0,-1 1 0,37-1 0,79 6 0,-61 0 0,-19-1 0,64 1 0,-118 0 0,0 0 0,-1 1 0,1-1 0,-1 1 0,1 1 0,-1-1 0,0 1 0,0 0 0,0 1 0,11 7 0,-2 2 0,1 1 0,16 21 0,-25-28 0,5 9 0,0 0 0,-1 1 0,12 25 0,10 16 0,-27-47 0,0 0 0,0 1 0,-2 1 0,1-1 0,-2 0 0,1 0 0,-2 1 0,3 22 0,7 22 0,-7-36 0,4 32 0,-5 1 0,-2-1 0,-7 59 0,4-101 0,-2-1 0,1 0 0,-1-1 0,-1 1 0,0 0 0,0 0 0,-1-1 0,-11 16 0,11-17 0,1-1 0,-1-1 0,0 0 0,0 0 0,-1-1 0,1 1 0,-1-1 0,0 0 0,-8 4 0,-5 2 0,-33 16 0,24-17 0,0-1 0,0-1 0,-56 9 0,30-12 0,-88-3 0,87-3 0,28-2-338,0 0-1,0-2 0,0-1 1,-37-14-1,-12-1-162,33 8 429,-39-6 509,1-2 1283,57 15-2976,3 1-5570</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1579.38">720 1659 24575,'0'-14'0,"0"1"0,1 0 0,0 0 0,1-1 0,0 1 0,1 1 0,1-2 0,0 2 0,1 0 0,10-21 0,-1 11 0,31-40 0,-9 14 0,-20 28 0,0 0 0,3 1 0,29-26 0,65-44 0,-107 85 0,139-88-685,-108 69 781,87-40-96,-122 62 14,1-1-1,0 1 1,0-1 0,0 1 0,-1 0-1,1 0 1,0 1 0,0-1-1,4 0 1,-6 1 3,0 0 1,1 0-1,-1 1 0,0-1 1,0 0-1,0 1 1,1-1-1,-1 1 0,0-1 1,0 1-1,0 0 1,0-1-1,0 1 0,0 0 1,0 0-1,0 0 1,0-1-1,-1 1 0,1 0 1,0 0-1,0 0 1,-1 1-1,1-1 0,-1 0 1,2 2-1,4 13-17,0 1 0,0 0 0,-2 0 0,0 0 0,0 0 0,0 24 0,-2 111 0,-3-101 0,0-34 0,-1 0 0,-1 0 0,-7 24 0,5-19 0,-4 26 0,-7 35 0,10-58 0,2 0 0,-3 29 0,5-18 0,3 43 0,1-67 0,-1 1 0,1-1 0,1 0 0,0-1 0,1 2 0,0-2 0,7 14 0,2 3 0,9 28 0,-13-29 0,23 41 0,-22-49 0,-3-6 0,-1-1 0,2 1 0,0-2 0,0 0 0,19 20 0,-27-30 0,0-1 0,1 1 0,-1-1 0,1 1 0,0 0 0,-1-1 0,1 0 0,-1 1 0,1-1 0,0 1 0,-1-1 0,1 0 0,0 1 0,-1-1 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 1 0,0-1 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1-1 0,1 1 0,0 0 0,-1 0 0,1 0 0,0-1 0,0 1 0,0-1 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0-2 0,0 2 0,-1-2 0,-6-34 0,-16-54 0,-9-10 0,16 57-64,4 6-586,-21-39-1,24 58-6175</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2028.66">875 1309 24575,'11'1'0,"0"0"0,0 1 0,-1 1 0,0 0 0,11 4 0,2 2 0,73 23 0,-18 0 0,2 1 0,-49-23-341,0-2 0,0-2-1,55 6 1,-59-10-6485</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2525.38">1779 1309 24575,'0'27'0,"0"-3"0,0 0 0,-1 0 0,-1 0 0,-7 29 0,2-22 13,1 0 1,-2 60-1,8 66-208,2-69-1015,-2-61-5616</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -5269,10 +5645,10 @@
       <inkml:brushProperty name="height" value="0.035" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">92 252 24575,'0'6'0,"0"6"0,0 7 0,0 6 0,0 3 0,0 3 0,0 1 0,0 0 0,0 0 0,0 1 0,0-1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 0 0,0-5-8191</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1556.43">29 128 24575,'4'-1'0,"-1"0"0,1 0 0,-1 0 0,0-1 0,1 1 0,-1-1 0,4-3 0,4-1 0,7-3 0,-8 4 0,0 0 0,1 0 0,0 1 0,15-4 0,26-4 0,-13 3 0,54-6 0,-66 12 0,36-10 0,-39 7 0,51-5 0,-64 10 0,7 0 0,-1 1 0,1 0 0,18 3 0,-31-3 0,0 1 0,-1 0 0,1 1 0,0-1 0,-1 1 0,1 0 0,-1 0 0,0 0 0,1 1 0,-1-1 0,0 1 0,0 0 0,-1 0 0,1 1 0,5 6 0,4 6 0,-5-7 0,-1 1 0,-1-1 0,1 1 0,-1 0 0,5 13 0,-2 0 0,0 0 0,-2 1 0,0 0 0,-2 0 0,4 43 0,-9 33 0,-1-86 0,-1 1 0,0-1 0,-1 0 0,-9 27 0,10-38 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,0-1 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,-1 0 0,1-1 0,-1 1 0,1-1 0,-1 0 0,1 0 0,-1 0 0,-5 1 0,-9 0 0,0-1 0,0 0 0,-28-3 0,21 0 0,-60 2 0,-51-4 0,122 1 12,-1 0 1,1-1-1,-1 0 0,1-1 0,1-1 0,-1 0 0,-16-11 1,-39-16-1476,49 26-5363</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2514.8">122 812 24575,'0'6'0,"0"6"0,0 7 0,0 6 0,0 3 0,0 3 0,0 1 0,0 0 0,0 1 0,0-1 0,-5-5 0,-2-3 0,0 1 0,2 1 0,-4-4 0,-1-1 0,2-3-8191</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="4045.87">60 626 24575,'0'376'0,"-1"-357"0,-1 1 0,-1 0 0,-6 21 0,3-18 0,-3 41 0,7-28 0,2-17 0,-1 1 0,-1 0 0,-7 27 0,-3 3-1365,8-27-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">92 259 24575,'0'6'0,"0"6"0,0 8 0,0 5 0,0 4 0,0 3 0,0 1 0,0-1 0,0 1 0,0 1 0,0-1 0,0-1 0,0 1 0,0-1 0,0-1 0,0 1 0,0-5-8191</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1556.43">29 131 24575,'4'-1'0,"-1"0"0,1 0 0,-1 0 0,0-1 0,1 1 0,-1-1 0,4-3 0,4-1 0,7-3 0,-8 3 0,0 1 0,1 0 0,0 1 0,15-4 0,26-4 0,-13 2 0,54-5 0,-66 12 0,36-10 0,-39 6 0,51-4 0,-64 10 0,7 0 0,-1 1 0,1 0 0,18 3 0,-31-3 0,0 1 0,-1 0 0,1 1 0,0-1 0,-1 1 0,1 0 0,-1 0 0,0 0 0,1 2 0,-1-2 0,0 1 0,0 0 0,-1 0 0,1 1 0,5 6 0,4 7 0,-5-8 0,-1 1 0,-1-1 0,1 2 0,-1-1 0,5 13 0,-2 1 0,0 0 0,-2 0 0,0 1 0,-2 0 0,4 43 0,-9 35 0,-1-89 0,-1 2 0,0-2 0,-1 0 0,-9 29 0,10-40 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,-1 0 0,1-1 0,-1 1 0,1-1 0,-1 0 0,1 0 0,-1 0 0,-5 1 0,-9 0 0,0-1 0,0 0 0,-28-3 0,21 0 0,-60 2 0,-51-4 0,122 1 12,-1 0 1,1-1-1,-1-1 0,1 0 0,1-1 0,-1 0 0,-16-11 1,-39-17-1476,49 26-5363</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2514.8">122 833 24575,'0'7'0,"0"5"0,0 7 0,0 7 0,0 3 0,0 3 0,0 0 0,0 1 0,0 1 0,0-1 0,-5-5 0,-2-4 0,0 2 0,2 1 0,-4-5 0,-1 0 0,2-4-8191</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="4045.87">60 642 24575,'0'386'0,"-1"-366"0,-1 0 0,-1 1 0,-6 21 0,3-18 0,-3 41 0,7-28 0,2-17 0,-1 0 0,-1 1 0,-7 27 0,-3 3-1365,8-27-5461</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -5299,7 +5675,7 @@
       <inkml:brushProperty name="height" value="0.035" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">188 1 24575,'0'442'-3597,"2"-414"3597,1 0 0,10 47 0,-1-17 0,-4-13-158,2 15-853,5 73 1,-14-64 544,0-14 481,10 65 0,6 80-15,-14-134 0,10 46-890,0 4-835,-8 319 1255,-7-244-1199,2 188 1719,-2-347-50,-1 0 0,-7 31 0,-3 25 0,10-65 403,-10 37-1,7-36-23,-4 33 0,-11 51-379,10-61 0,-2-2 0,8-29 0,-4 21 0,-26 145 625,22-118-625,5-32 0,-4 61 0,9-69 0,0-1 0,-1 0 0,-2 0 0,-15 42 0,15-46 0,1 0 0,1 1 0,0 0 0,0 24 0,2 80 3,1 0-51,-13-27-198,7-65 254,-1 35 1,5 209 925,5-143-626,-2 369-308,-2-475-21,0 0 0,-9 38 0,4-32 182,-1 35 1,6 227 1018,3-151 1078,-1 202 1804,0-334-4101,1 0 0,0 0 0,1 0-1,0-1 1,1 1 0,8 21 0,-4-16-30,2 0 0,0-1 1,18 26-1,26 30 69,97 144 0,-127-179-95,20 32 304,-37-58-486,-1 0-1,0 0 1,-1 0-1,4 20 0,-4-8-6090</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">188 1 24575,'0'449'-3597,"3"-421"3597,0 0 0,10 48 0,-1-17 0,-4-13-158,2 15-853,5 74 1,-14-65 544,0-14 481,10 66 0,6 80-15,-14-135 0,10 47-890,0 4-835,-8 323 1255,-7-247-1199,2 191 1719,-2-353-50,-1 1 0,-7 31 0,-3 25 0,10-66 403,-10 38-1,7-36-23,-4 32 0,-11 53-379,10-62 0,-2-3 0,8-28 0,-4 20 0,-27 148 625,23-120-625,5-33 0,-4 63 0,9-71 0,0-1 0,-1 1 0,-2-1 0,-15 43 0,15-47 0,1 1 0,1 0 0,0 0 0,0 25 0,2 81 3,1-1-51,-13-26-198,7-67 254,-1 36 1,5 212 925,5-145-626,-2 375-308,-2-483-21,0 1 0,-9 38 0,4-33 182,-1 36 1,6 231 1018,3-154 1078,-1 205 1804,0-339-4101,1 0 0,0 0 0,1 0-1,0 0 1,1 0 0,8 21 0,-4-15-30,2-1 0,0-1 1,18 27-1,26 30 69,98 146 0,-128-181-95,20 32 304,-37-59-486,-1 0-1,0 0 1,-1 0-1,4 21 0,-4-9-6090</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -5326,11 +5702,11 @@
       <inkml:brushProperty name="height" value="0.035" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1396 33 24575,'1212'0'-2982,"-1191"-1"3016,-1-1-1,0-1 0,22-6 0,-18 4 1233,40-5 0,207 8-953,-139 4-309,-64-3-4,82 2 0,-127 2 0,25 7 0,5 1 0,34 6 0,-54-9 0,65 6 0,-12-14 0,13 1 0,-96-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,-1 1 0,1-1 0,-1 1 0,1 0 0,-1-1 0,0 1 0,0 0 0,0 0 0,0 5 0,2 7 0,-2 1 0,0-1 0,0 1 0,-4 24 0,2-17 0,0-4 0,1 3 0,-2 0 0,0 1 0,-10 40 0,-7 19 0,6-26 0,-3 12 0,-30 103 0,42-156 0,0 1 0,0-1 0,2 1 0,-1 17 0,2 63 0,0 7 0,-1-89 0,-1 0 0,-4 18 0,-3 10 0,-27 100 0,9-41 0,16-56 0,-23 56 0,14-36 0,-5 8 0,-16 55 205,6-17-2541,31-94 2225,0-1 0,2 1 0,0 0 0,-2 21 0,3-16 124,-9 39 0,5-35-16,1 1 0,1 0 1,0 29-1,4 82 62,1-66 216,0 695 1455,-2-747-1582,-1 0-1,-1 0 1,-6 21-1,3-17-138,-3 40-1,7-10-8,2-34 0,0 0 0,-2 1 0,0-1 0,-6 20 0,1-12 0,2 1 0,1 0 0,-1 34 0,6 89 0,0-63 0,-1-52 0,0-2 0,0 0 0,2 0 0,9 43 0,-3-36 0,-2 1 0,1 51 0,-7 89 0,-2-74 0,3-39 0,-3 80 0,-12-61 0,7-59 0,-2 40 0,7 205 0,4-142 0,-4-64 0,4 81 0,1-133 0,8 33 0,-6-33 0,4 29 0,-6-26 0,1 1 0,1-1 0,1 0 0,1 0 0,1 0 0,0-1 0,16 26 0,-7-11 0,23 63 0,-23-54 0,5 24 0,2 5 0,-16-50 0,-1 1 0,0 0 0,-2 0 0,-1 0 0,2 34 0,-5 120 0,-3-84 0,0-73 0,0 0 0,-1 0 0,-6 21 0,4-17 0,-4 40 0,8-57 0,1 0 0,-1 1 0,-1-1 0,1 0 0,-1-1 0,0 1 0,-1 0 0,-3 7 0,4-11 0,0 1 0,-1-1 0,1 1 0,-1-1 0,0 0 0,1 0 0,-2 0 0,1-1 0,0 1 0,0-1 0,-1 1 0,1-1 0,-1 0 0,0 0 0,-6 1 0,-1 1 0,-1-1 0,0-1 0,0 0 0,-20 0 0,-51-4 0,36 0 0,32 1-335,-1 1 0,0 1 0,0 1 0,0 0 0,-18 5 0,10-1 335,-1-1 0,1-1 0,-27 1 0,-76-4 0,86-2 0,24 2-249,0 1 1,1 0-1,-26 7 0,-25 4-358,-63 10 604,78-12 3,28-5 447,-44 17 0,46-14-133,0-2 0,-29 7 0,-73 17 310,89-21-340,0-1 0,-1-1 0,-45 3 1,55-9-281,-42 11 1,42-7 0,-42 3-1,-223-7-1619,147-4 1060,96 3 555,9 0 0,1-2 0,-1-1 0,-46-9 0,41 3-904,0 2-1,-49-1 0,-91 8-3415,81 0 3337,-474 0 1423,317-2 3064,233 1-5452</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1574.67">1210 3992 24575,'3'0'0,"-1"1"0,1 0 0,-1-1 0,0 1 0,0 0 0,1 0 0,-1 0 0,4 3 0,12 5 0,220 55-833,-147-52-364,5 1-89,-42-4 831,1-3 1,-1-2-1,63-4 0,-93 1 455,-1 1 0,40 9 0,14 2 0,21 3-154,-63-8 114,49 3 0,-39-9 1453,65-4-1,-94-1-992,-1-1 0,1 0 1,-1 0-1,20-10 0,25-7 23,-20 8-443,65-30 0,-15 10 0,-70 27-227,1 1-1,0 2 1,0 0-1,0 1 1,41 1-1,-35 1-6598</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2316.37">1490 3835 24575,'42'0'-31,"-17"-1"-40,0 1-1,1 1 1,-1 1 0,36 8-1,-28-3-316,-1-1 0,1-2 0,0-1 0,37-3-1,-43 2 72,0 0 0,38 10-1,-32-6-40,33 3-1,207-7 359,-141-4 0,428 2 0,-541-1 0,0-1 0,0-1 0,24-7 0,-21 5 0,43-5 0,-28 7 0,48-8 0,-54 5-699,-4 0-2795</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="3164.09">1957 4337 24575,'0'789'-3275,"1"-761"3275,2-1 0,8 38 0,-5-33 0,3 40 0,6 59-932,-7-82 382,1 50 0,-9 325 550,-1-196 0,1-202 0,-2 1 0,-8 53 0,2-37 14,2 1 0,0 65 0,6-25-2917,-3-23 1623,-2 0 0,-16 69 0,18-115 1226,-53 239-116,48-224 155,-40 196-145,39-155 509,-6 26-63,-1 15 139,1-5-30,-5 57 597,9-52-435,6-76-620,-21 133-305,19-112 681,-2 84 0,5-44-1192,-10 2 1867,-1 3 316,13 171-904,4-141-266,-2-115 256,0 0 0,1-1-1,1 1 1,7 29 0,-2-22 853,-1-3-5365</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="4207.75">2609 4212 24575,'0'1038'-3218,"-2"-1009"3218,0 0 0,-8 33 0,-4 26 0,-3 28-780,10-75 221,-4 67-1,9-68 214,-8 58-1,-28 149-2266,28-116 1912,6-51-741,2-65 1276,-8 30 0,0-2 160,6-24-65,-8 24 0,6-24 1464,-4 22 1,-20 75 2591,19-79-3263,-10 54 0,4-12-906,11-54 79,1-1 0,-4 39 0,7-7-292,2-26-400,-1 1 0,-8 39 0,-6 43 545,10-68 241,-9 36 1144,8-49-1019,-4 43 0,8 220-1528,4-149 925,-2 451 6075,0-347-5615,0-224-6797</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1397 33 24575,'1214'0'-2982,"-1193"-1"3016,-1-1-1,0-1 0,22-6 0,-18 4 1233,40-5 0,207 8-953,-139 4-309,-64-3-4,82 2 0,-127 2 0,25 7 0,6 1 0,33 7 0,-54-10 0,65 6 0,-12-14 0,13 1 0,-96-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,-1 1 0,1-1 0,-1 1 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 5 0,2 7 0,-2 1 0,0-1 0,0 2 0,-4 23 0,2-16 0,0-5 0,1 3 0,-2 0 0,0 2 0,-10 40 0,-7 19 0,6-26 0,-3 11 0,-30 106 0,42-159 0,0 1 0,0 0 0,2 0 0,-1 17 0,2 65 0,0 6 0,-1-90 0,-1 0 0,-4 19 0,-3 9 0,-27 102 0,9-41 0,16-57 0,-23 56 0,14-36 0,-5 8 0,-16 56 205,6-18-2541,31-95 2225,0 0 0,2 0 0,0 0 0,-2 22 0,3-17 124,-9 40 0,5-36-16,1 2 0,1-1 1,0 30-1,4 83 62,1-67 216,0 704 1455,-2-756-1582,-1-1-1,-1 0 1,-6 22-1,3-18-138,-3 41-1,7-10-8,2-35 0,0 0 0,-2 2 0,0-2 0,-6 21 0,1-13 0,2 1 0,0 1 0,0 34 0,6 90 0,0-64 0,-1-52 0,0-3 0,0 1 0,2-1 0,10 44 0,-4-36 0,-2 0 0,1 53 0,-7 89 0,-2-74 0,3-40 0,-3 81 0,-12-62 0,7-59 0,-3 40 0,8 207 0,4-143 0,-4-65 0,4 82 0,1-134 0,9 32 0,-7-32 0,4 28 0,-6-26 0,1 2 0,1-2 0,1 0 0,1 1 0,1-1 0,0-1 0,16 27 0,-7-12 0,23 65 0,-23-56 0,5 25 0,2 5 0,-16-51 0,-1 2 0,0-1 0,-2 0 0,-1 1 0,2 34 0,-5 121 0,-3-85 0,0-73 0,0-1 0,-1 0 0,-6 22 0,4-18 0,-4 41 0,8-58 0,1 0 0,-1 1 0,-1-1 0,1 1 0,-1-2 0,0 1 0,-1 0 0,-3 7 0,4-11 0,0 1 0,-1-1 0,1 1 0,-1-1 0,0 0 0,1 0 0,-2 0 0,1-1 0,0 1 0,0-1 0,-1 1 0,1 0 0,-1-1 0,0 0 0,-6 1 0,-1 1 0,-1-1 0,0-1 0,0 0 0,-20 0 0,-52-4 0,37 0 0,32 1-335,-1 1 0,0 1 0,0 1 0,0 0 0,-18 5 0,10-1 335,-1-1 0,1-1 0,-27 1 0,-76-4 0,86-2 0,24 2-249,0 1 1,1 0-1,-26 7 0,-25 5-358,-63 9 604,78-12 3,28-5 447,-44 17 0,46-13-133,0-3 0,-29 7 0,-74 17 310,90-21-340,0 0 0,-1-2 0,-45 3 1,55-9-281,-42 11 1,42-7 0,-42 3-1,-223-7-1619,147-4 1060,96 3 555,8 0 0,2-2 0,-1-1 0,-46-9 0,41 3-904,0 2-1,-49-1 0,-91 8-3415,81 0 3337,-475 0 1423,318-2 3064,233 1-5452</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1574.66">1211 4048 24575,'3'0'0,"-1"1"0,1 0 0,-1-1 0,0 1 0,0 0 0,1 0 0,-1 0 0,4 3 0,12 5 0,220 56-833,-146-53-364,4 2-89,-42-5 831,1-3 1,-1-2-1,63-4 0,-93 1 455,-1 1 0,40 9 0,14 2 0,21 3-154,-63-7 114,49 2 0,-39-9 1453,66-4-1,-95-1-992,-1-1 0,1 0 1,-1 0-1,20-11 0,25-6 23,-20 8-443,65-31 0,-15 11 0,-70 27-227,1 1-1,0 2 1,0 0-1,0 0 1,41 2-1,-35 1-6598</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2316.37">1491 3889 24575,'43'0'-31,"-18"-1"-40,0 1-1,1 1 1,-1 1 0,36 8-1,-28-3-316,-1-1 0,1-2 0,0-1 0,37-3-1,-43 2 72,0 0 0,38 11-1,-32-7-40,33 3-1,207-7 359,-140-4 0,427 2 0,-541-1 0,0-1 0,0-1 0,24-7 0,-21 4 0,43-4 0,-28 7 0,48-8 0,-54 5-699,-4 0-2795</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="3164.09">1959 4398 24575,'0'800'-3275,"1"-772"3275,2 0 0,8 38 0,-5-34 0,3 41 0,6 60-932,-7-83 382,1 50 0,-9 330 550,-1-199 0,1-204 0,-2 0 0,-8 54 0,2-37 14,2 0 0,0 67 0,6-26-2917,-3-23 1623,-2 0 0,-16 70 0,18-117 1226,-53 242-116,48-226 155,-40 198-145,39-157 509,-6 26-63,-1 16 139,1-6-30,-5 59 597,9-54-435,6-76-620,-21 134-305,19-113 681,-2 85 0,5-45-1192,-10 3 1867,-1 2 316,13 174-904,4-143-266,-2-117 256,0 0 0,1-1-1,1 2 1,7 28 0,-2-21 853,-1-4-5365</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="4207.75">2612 4271 24575,'0'1053'-3218,"-2"-1024"3218,0 1 0,-8 32 0,-4 28 0,-3 27-780,10-75 221,-4 67-1,9-68 214,-8 58-1,-29 152-2266,29-118 1912,6-52-741,2-66 1276,-8 31 0,0-3 160,6-24-65,-8 25 0,6-25 1464,-4 23 1,-20 76 2591,19-81-3263,-10 55 0,4-12-906,11-54 79,1-2 0,-4 40 0,7-7-292,2-27-400,-1 2 0,-8 39 0,-6 43 545,10-68 241,-9 36 1144,8-50-1019,-4 44 0,8 224-1528,4-152 925,-2 457 6075,0-351-5615,0-228-6797</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -5732,7 +6108,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B349714-3586-4A93-AA4E-11E81A6892D2}">
-  <dimension ref="A1:J85"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="23.6640625" customWidth="1"/>
@@ -6277,9 +6653,6 @@
       </c>
       <c r="E55" s="7"/>
     </row>
-    <row r="85" spans="10:10" x14ac:dyDescent="0.45">
-      <c r="J85" s="10"/>
-    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="B1:D1"/>

</xml_diff>